<commit_message>
fix(frontend): booked-cell popup resolves Name-<ID> via student_id\n\n- Parse trailing numeric token after '-' and search by student_id first\n- Rebuild frontend assets and update index.html\n- Update Excel test data
</commit_message>
<xml_diff>
--- a/api/data/Test.xlsx
+++ b/api/data/Test.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3438" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3438" uniqueCount="26">
   <si>
     <t>AM</t>
   </si>
@@ -69,6 +69,12 @@
   </si>
   <si>
     <t>Dhwani Patel [SID:139582853530]</t>
+  </si>
+  <si>
+    <t>Ibrahim Mohamed [SID:113611046408]</t>
+  </si>
+  <si>
+    <t>Ibrahim Mohamed-2401841</t>
   </si>
   <si>
     <t>Lab B</t>
@@ -919,10 +925,10 @@
         <v>17</v>
       </c>
       <c r="M7" s="7" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" ht="19.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -936,10 +942,10 @@
         <v>8</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>8</v>
@@ -2379,7 +2385,7 @@
     </row>
     <row r="41" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B41" s="14">
         <v>1</v>
@@ -2423,7 +2429,7 @@
     </row>
     <row r="42" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B42" s="14">
         <v>2</v>
@@ -2467,7 +2473,7 @@
     </row>
     <row r="43" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B43" s="14">
         <v>3</v>
@@ -2511,7 +2517,7 @@
     </row>
     <row r="44" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B44" s="14">
         <v>4</v>
@@ -2555,7 +2561,7 @@
     </row>
     <row r="45" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B45" s="14">
         <v>5</v>
@@ -2599,7 +2605,7 @@
     </row>
     <row r="46" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B46" s="14">
         <v>6</v>
@@ -2643,7 +2649,7 @@
     </row>
     <row r="47" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B47" s="14">
         <v>7</v>
@@ -2687,7 +2693,7 @@
     </row>
     <row r="48" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B48" s="14">
         <v>8</v>
@@ -2731,7 +2737,7 @@
     </row>
     <row r="49" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B49" s="14">
         <v>9</v>
@@ -2775,7 +2781,7 @@
     </row>
     <row r="50" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B50" s="14">
         <v>10</v>
@@ -2819,7 +2825,7 @@
     </row>
     <row r="51" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B51" s="14">
         <v>11</v>
@@ -2863,7 +2869,7 @@
     </row>
     <row r="52" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B52" s="14">
         <v>12</v>
@@ -2907,7 +2913,7 @@
     </row>
     <row r="53" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B53" s="14">
         <v>13</v>
@@ -2951,7 +2957,7 @@
     </row>
     <row r="54" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B54" s="14">
         <v>14</v>
@@ -2995,7 +3001,7 @@
     </row>
     <row r="55" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B55" s="14">
         <v>15</v>
@@ -3039,7 +3045,7 @@
     </row>
     <row r="56" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B56" s="14">
         <v>16</v>
@@ -3083,7 +3089,7 @@
     </row>
     <row r="57" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B57" s="14">
         <v>17</v>
@@ -3127,7 +3133,7 @@
     </row>
     <row r="58" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B58" s="14">
         <v>18</v>
@@ -3171,7 +3177,7 @@
     </row>
     <row r="59" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B59" s="14">
         <v>19</v>
@@ -3215,7 +3221,7 @@
     </row>
     <row r="60" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B60" s="14">
         <v>20</v>
@@ -3259,7 +3265,7 @@
     </row>
     <row r="61" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A61" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B61" s="14">
         <v>21</v>
@@ -3303,7 +3309,7 @@
     </row>
     <row r="62" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B62" s="14">
         <v>22</v>
@@ -3347,7 +3353,7 @@
     </row>
     <row r="63" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A63" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B63" s="14">
         <v>23</v>
@@ -3391,7 +3397,7 @@
     </row>
     <row r="64" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B64" s="14">
         <v>24</v>
@@ -3435,7 +3441,7 @@
     </row>
     <row r="65" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B65" s="14">
         <v>25</v>
@@ -3479,7 +3485,7 @@
     </row>
     <row r="66" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B66" s="14">
         <v>26</v>
@@ -3523,7 +3529,7 @@
     </row>
     <row r="67" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A67" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B67" s="14">
         <v>27</v>
@@ -3567,7 +3573,7 @@
     </row>
     <row r="68" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B68" s="14">
         <v>28</v>
@@ -3611,7 +3617,7 @@
     </row>
     <row r="69" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A69" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B69" s="14">
         <v>29</v>
@@ -3655,7 +3661,7 @@
     </row>
     <row r="70" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B70" s="14">
         <v>30</v>
@@ -3699,7 +3705,7 @@
     </row>
     <row r="71" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A71" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B71" s="14">
         <v>31</v>
@@ -3743,7 +3749,7 @@
     </row>
     <row r="72" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A72" s="13" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B72" s="14">
         <v>1</v>
@@ -3787,7 +3793,7 @@
     </row>
     <row r="73" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B73" s="14">
         <v>2</v>
@@ -3831,7 +3837,7 @@
     </row>
     <row r="74" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A74" s="13" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B74" s="14">
         <v>3</v>
@@ -3875,7 +3881,7 @@
     </row>
     <row r="75" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B75" s="14">
         <v>4</v>
@@ -3919,7 +3925,7 @@
     </row>
     <row r="76" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A76" s="13" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B76" s="14">
         <v>5</v>
@@ -3963,7 +3969,7 @@
     </row>
     <row r="77" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B77" s="14">
         <v>6</v>
@@ -4007,7 +4013,7 @@
     </row>
     <row r="78" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A78" s="13" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B78" s="14">
         <v>7</v>
@@ -4051,7 +4057,7 @@
     </row>
     <row r="79" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B79" s="14">
         <v>8</v>
@@ -4095,7 +4101,7 @@
     </row>
     <row r="80" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A80" s="13" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B80" s="14">
         <v>9</v>
@@ -4139,7 +4145,7 @@
     </row>
     <row r="81" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B81" s="14">
         <v>10</v>
@@ -4183,7 +4189,7 @@
     </row>
     <row r="82" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A82" s="13" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B82" s="14">
         <v>11</v>
@@ -4227,7 +4233,7 @@
     </row>
     <row r="83" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B83" s="14">
         <v>12</v>
@@ -4271,7 +4277,7 @@
     </row>
     <row r="84" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A84" s="13" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B84" s="14">
         <v>13</v>
@@ -4315,7 +4321,7 @@
     </row>
     <row r="85" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B85" s="14">
         <v>14</v>
@@ -4359,7 +4365,7 @@
     </row>
     <row r="86" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A86" s="13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B86" s="14">
         <v>1</v>
@@ -4403,7 +4409,7 @@
     </row>
     <row r="87" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B87" s="14">
         <v>2</v>
@@ -4447,7 +4453,7 @@
     </row>
     <row r="88" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A88" s="13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B88" s="14">
         <v>3</v>
@@ -4491,7 +4497,7 @@
     </row>
     <row r="89" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B89" s="14">
         <v>4</v>
@@ -4535,7 +4541,7 @@
     </row>
     <row r="90" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A90" s="13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B90" s="14">
         <v>5</v>
@@ -4579,7 +4585,7 @@
     </row>
     <row r="91" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B91" s="14">
         <v>6</v>
@@ -4623,7 +4629,7 @@
     </row>
     <row r="92" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A92" s="13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B92" s="14">
         <v>7</v>
@@ -4667,7 +4673,7 @@
     </row>
     <row r="93" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B93" s="14">
         <v>8</v>
@@ -4711,7 +4717,7 @@
     </row>
     <row r="94" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A94" s="13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B94" s="14">
         <v>9</v>
@@ -4755,7 +4761,7 @@
     </row>
     <row r="95" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B95" s="14">
         <v>10</v>
@@ -4799,7 +4805,7 @@
     </row>
     <row r="96" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A96" s="13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B96" s="14">
         <v>11</v>
@@ -4843,7 +4849,7 @@
     </row>
     <row r="97" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B97" s="14">
         <v>12</v>
@@ -4887,7 +4893,7 @@
     </row>
     <row r="98" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A98" s="13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B98" s="14">
         <v>13</v>
@@ -4931,7 +4937,7 @@
     </row>
     <row r="99" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B99" s="14">
         <v>14</v>
@@ -4975,7 +4981,7 @@
     </row>
     <row r="100" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A100" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B100" s="17">
         <v>1</v>
@@ -5019,7 +5025,7 @@
     </row>
     <row r="101" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A101" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B101" s="17">
         <v>2</v>
@@ -5063,7 +5069,7 @@
     </row>
     <row r="102" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A102" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B102" s="17">
         <v>3</v>
@@ -5107,7 +5113,7 @@
     </row>
     <row r="103" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A103" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B103" s="17">
         <v>4</v>
@@ -5151,7 +5157,7 @@
     </row>
     <row r="104" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A104" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B104" s="17">
         <v>5</v>
@@ -5195,7 +5201,7 @@
     </row>
     <row r="105" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A105" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B105" s="17">
         <v>6</v>
@@ -5239,7 +5245,7 @@
     </row>
     <row r="106" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A106" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B106" s="17">
         <v>7</v>
@@ -5283,7 +5289,7 @@
     </row>
     <row r="107" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A107" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B107" s="17">
         <v>8</v>
@@ -5327,7 +5333,7 @@
     </row>
     <row r="108" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A108" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B108" s="17">
         <v>9</v>
@@ -5371,7 +5377,7 @@
     </row>
     <row r="109" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A109" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B109" s="17">
         <v>10</v>
@@ -5415,7 +5421,7 @@
     </row>
     <row r="110" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A110" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B110" s="17">
         <v>11</v>
@@ -5459,7 +5465,7 @@
     </row>
     <row r="111" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A111" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B111" s="17">
         <v>12</v>
@@ -5503,7 +5509,7 @@
     </row>
     <row r="112" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A112" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B112" s="17">
         <v>13</v>
@@ -5547,7 +5553,7 @@
     </row>
     <row r="113" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A113" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B113" s="17">
         <v>14</v>
@@ -5591,7 +5597,7 @@
     </row>
     <row r="114" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A114" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B114" s="17">
         <v>15</v>
@@ -5635,7 +5641,7 @@
     </row>
     <row r="115" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A115" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B115" s="17">
         <v>16</v>
@@ -5679,7 +5685,7 @@
     </row>
     <row r="116" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A116" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B116" s="17">
         <v>17</v>
@@ -5723,7 +5729,7 @@
     </row>
     <row r="117" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A117" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B117" s="17">
         <v>18</v>
@@ -5767,7 +5773,7 @@
     </row>
     <row r="118" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A118" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B118" s="17">
         <v>19</v>
@@ -5811,7 +5817,7 @@
     </row>
     <row r="119" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A119" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B119" s="17">
         <v>20</v>
@@ -5855,7 +5861,7 @@
     </row>
     <row r="120" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A120" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B120" s="23">
         <v>1</v>
@@ -5899,7 +5905,7 @@
     </row>
     <row r="121" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A121" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B121" s="24">
         <v>2</v>
@@ -5943,7 +5949,7 @@
     </row>
     <row r="122" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A122" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B122" s="23">
         <v>3</v>
@@ -5987,7 +5993,7 @@
     </row>
     <row r="123" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A123" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B123" s="24">
         <v>4</v>
@@ -6031,7 +6037,7 @@
     </row>
     <row r="124" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A124" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B124" s="23">
         <v>5</v>
@@ -6075,7 +6081,7 @@
     </row>
     <row r="125" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A125" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B125" s="24">
         <v>6</v>
@@ -6119,7 +6125,7 @@
     </row>
     <row r="126" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A126" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B126" s="23">
         <v>7</v>
@@ -6163,7 +6169,7 @@
     </row>
     <row r="127" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A127" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B127" s="24">
         <v>8</v>
@@ -6207,7 +6213,7 @@
     </row>
     <row r="128" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A128" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B128" s="23">
         <v>9</v>
@@ -6251,7 +6257,7 @@
     </row>
     <row r="129" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A129" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B129" s="24">
         <v>10</v>
@@ -6295,7 +6301,7 @@
     </row>
     <row r="130" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A130" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B130" s="23">
         <v>11</v>
@@ -6339,7 +6345,7 @@
     </row>
     <row r="131" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A131" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B131" s="24">
         <v>12</v>
@@ -6383,7 +6389,7 @@
     </row>
     <row r="132" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A132" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B132" s="23">
         <v>13</v>
@@ -6427,7 +6433,7 @@
     </row>
     <row r="133" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A133" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B133" s="24">
         <v>14</v>
@@ -6471,7 +6477,7 @@
     </row>
     <row r="134" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A134" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B134" s="23">
         <v>15</v>
@@ -19523,7 +19529,7 @@
   <sheetData>
     <row r="1" ht="18" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4">
@@ -21281,7 +21287,7 @@
     </row>
     <row r="41" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B41" s="14">
         <v>1</v>
@@ -21325,7 +21331,7 @@
     </row>
     <row r="42" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B42" s="14">
         <v>2</v>
@@ -21369,7 +21375,7 @@
     </row>
     <row r="43" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B43" s="14">
         <v>3</v>
@@ -21413,7 +21419,7 @@
     </row>
     <row r="44" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B44" s="14">
         <v>4</v>
@@ -21457,7 +21463,7 @@
     </row>
     <row r="45" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B45" s="14">
         <v>5</v>
@@ -21501,7 +21507,7 @@
     </row>
     <row r="46" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B46" s="14">
         <v>6</v>
@@ -21545,7 +21551,7 @@
     </row>
     <row r="47" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B47" s="14">
         <v>7</v>
@@ -21589,7 +21595,7 @@
     </row>
     <row r="48" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B48" s="14">
         <v>8</v>
@@ -21633,7 +21639,7 @@
     </row>
     <row r="49" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B49" s="14">
         <v>9</v>
@@ -21677,7 +21683,7 @@
     </row>
     <row r="50" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B50" s="14">
         <v>10</v>
@@ -21721,7 +21727,7 @@
     </row>
     <row r="51" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B51" s="14">
         <v>11</v>
@@ -21765,7 +21771,7 @@
     </row>
     <row r="52" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B52" s="14">
         <v>12</v>
@@ -21809,7 +21815,7 @@
     </row>
     <row r="53" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B53" s="14">
         <v>13</v>
@@ -21853,7 +21859,7 @@
     </row>
     <row r="54" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B54" s="14">
         <v>14</v>
@@ -21897,7 +21903,7 @@
     </row>
     <row r="55" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B55" s="14">
         <v>15</v>
@@ -21941,7 +21947,7 @@
     </row>
     <row r="56" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B56" s="14">
         <v>16</v>
@@ -21985,7 +21991,7 @@
     </row>
     <row r="57" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B57" s="14">
         <v>17</v>
@@ -22029,7 +22035,7 @@
     </row>
     <row r="58" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B58" s="14">
         <v>18</v>
@@ -22073,7 +22079,7 @@
     </row>
     <row r="59" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A59" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B59" s="14">
         <v>19</v>
@@ -22117,7 +22123,7 @@
     </row>
     <row r="60" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B60" s="14">
         <v>20</v>
@@ -22161,7 +22167,7 @@
     </row>
     <row r="61" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A61" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B61" s="14">
         <v>21</v>
@@ -22205,7 +22211,7 @@
     </row>
     <row r="62" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B62" s="14">
         <v>22</v>
@@ -22249,7 +22255,7 @@
     </row>
     <row r="63" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A63" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B63" s="14">
         <v>23</v>
@@ -22293,7 +22299,7 @@
     </row>
     <row r="64" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B64" s="14">
         <v>24</v>
@@ -22337,7 +22343,7 @@
     </row>
     <row r="65" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B65" s="14">
         <v>25</v>
@@ -22381,7 +22387,7 @@
     </row>
     <row r="66" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B66" s="14">
         <v>26</v>
@@ -22425,7 +22431,7 @@
     </row>
     <row r="67" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A67" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B67" s="14">
         <v>27</v>
@@ -22469,7 +22475,7 @@
     </row>
     <row r="68" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B68" s="14">
         <v>28</v>
@@ -22513,7 +22519,7 @@
     </row>
     <row r="69" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A69" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B69" s="14">
         <v>29</v>
@@ -22557,7 +22563,7 @@
     </row>
     <row r="70" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B70" s="14">
         <v>30</v>
@@ -22601,7 +22607,7 @@
     </row>
     <row r="71" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A71" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B71" s="14">
         <v>31</v>
@@ -22645,7 +22651,7 @@
     </row>
     <row r="72" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A72" s="13" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B72" s="14">
         <v>1</v>
@@ -22689,7 +22695,7 @@
     </row>
     <row r="73" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B73" s="14">
         <v>2</v>
@@ -22733,7 +22739,7 @@
     </row>
     <row r="74" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A74" s="13" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B74" s="14">
         <v>3</v>
@@ -22777,7 +22783,7 @@
     </row>
     <row r="75" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B75" s="14">
         <v>4</v>
@@ -22821,7 +22827,7 @@
     </row>
     <row r="76" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A76" s="13" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B76" s="14">
         <v>5</v>
@@ -22865,7 +22871,7 @@
     </row>
     <row r="77" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B77" s="14">
         <v>6</v>
@@ -22909,7 +22915,7 @@
     </row>
     <row r="78" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A78" s="13" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B78" s="14">
         <v>7</v>
@@ -22953,7 +22959,7 @@
     </row>
     <row r="79" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B79" s="14">
         <v>8</v>
@@ -22997,7 +23003,7 @@
     </row>
     <row r="80" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A80" s="13" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B80" s="14">
         <v>9</v>
@@ -23041,7 +23047,7 @@
     </row>
     <row r="81" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B81" s="14">
         <v>10</v>
@@ -23085,7 +23091,7 @@
     </row>
     <row r="82" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A82" s="13" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B82" s="14">
         <v>11</v>
@@ -23129,7 +23135,7 @@
     </row>
     <row r="83" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B83" s="14">
         <v>12</v>
@@ -23173,7 +23179,7 @@
     </row>
     <row r="84" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A84" s="13" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B84" s="14">
         <v>13</v>
@@ -23217,7 +23223,7 @@
     </row>
     <row r="85" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B85" s="14">
         <v>14</v>
@@ -23261,7 +23267,7 @@
     </row>
     <row r="86" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A86" s="13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B86" s="14">
         <v>1</v>
@@ -23305,7 +23311,7 @@
     </row>
     <row r="87" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B87" s="14">
         <v>2</v>
@@ -23349,7 +23355,7 @@
     </row>
     <row r="88" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A88" s="13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B88" s="14">
         <v>3</v>
@@ -23393,7 +23399,7 @@
     </row>
     <row r="89" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B89" s="14">
         <v>4</v>
@@ -23437,7 +23443,7 @@
     </row>
     <row r="90" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A90" s="13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B90" s="14">
         <v>5</v>
@@ -23481,7 +23487,7 @@
     </row>
     <row r="91" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B91" s="14">
         <v>6</v>
@@ -23525,7 +23531,7 @@
     </row>
     <row r="92" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A92" s="13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B92" s="14">
         <v>7</v>
@@ -23569,7 +23575,7 @@
     </row>
     <row r="93" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B93" s="14">
         <v>8</v>
@@ -23613,7 +23619,7 @@
     </row>
     <row r="94" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A94" s="13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B94" s="14">
         <v>9</v>
@@ -23657,7 +23663,7 @@
     </row>
     <row r="95" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B95" s="14">
         <v>10</v>
@@ -23701,7 +23707,7 @@
     </row>
     <row r="96" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A96" s="13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B96" s="14">
         <v>11</v>
@@ -23745,7 +23751,7 @@
     </row>
     <row r="97" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B97" s="14">
         <v>12</v>
@@ -23789,7 +23795,7 @@
     </row>
     <row r="98" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A98" s="13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B98" s="14">
         <v>13</v>
@@ -23833,7 +23839,7 @@
     </row>
     <row r="99" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B99" s="14">
         <v>14</v>
@@ -23877,7 +23883,7 @@
     </row>
     <row r="100" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A100" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B100" s="17">
         <v>1</v>
@@ -23921,7 +23927,7 @@
     </row>
     <row r="101" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A101" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B101" s="17">
         <v>2</v>
@@ -23965,7 +23971,7 @@
     </row>
     <row r="102" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A102" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B102" s="17">
         <v>3</v>
@@ -24009,7 +24015,7 @@
     </row>
     <row r="103" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A103" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B103" s="17">
         <v>4</v>
@@ -24053,7 +24059,7 @@
     </row>
     <row r="104" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A104" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B104" s="17">
         <v>5</v>
@@ -24097,7 +24103,7 @@
     </row>
     <row r="105" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A105" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B105" s="17">
         <v>6</v>
@@ -24141,7 +24147,7 @@
     </row>
     <row r="106" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A106" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B106" s="17">
         <v>7</v>
@@ -24185,7 +24191,7 @@
     </row>
     <row r="107" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A107" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B107" s="17">
         <v>8</v>
@@ -24229,7 +24235,7 @@
     </row>
     <row r="108" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A108" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B108" s="17">
         <v>9</v>
@@ -24273,7 +24279,7 @@
     </row>
     <row r="109" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A109" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B109" s="17">
         <v>10</v>
@@ -24317,7 +24323,7 @@
     </row>
     <row r="110" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A110" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B110" s="17">
         <v>11</v>
@@ -24361,7 +24367,7 @@
     </row>
     <row r="111" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A111" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B111" s="17">
         <v>12</v>
@@ -24405,7 +24411,7 @@
     </row>
     <row r="112" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A112" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B112" s="17">
         <v>13</v>
@@ -24449,7 +24455,7 @@
     </row>
     <row r="113" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A113" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B113" s="17">
         <v>14</v>
@@ -24493,7 +24499,7 @@
     </row>
     <row r="114" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A114" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B114" s="17">
         <v>15</v>
@@ -24537,7 +24543,7 @@
     </row>
     <row r="115" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A115" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B115" s="17">
         <v>16</v>
@@ -24581,7 +24587,7 @@
     </row>
     <row r="116" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A116" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B116" s="17">
         <v>17</v>
@@ -24625,7 +24631,7 @@
     </row>
     <row r="117" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A117" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B117" s="17">
         <v>18</v>
@@ -24669,7 +24675,7 @@
     </row>
     <row r="118" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A118" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B118" s="17">
         <v>19</v>
@@ -24713,7 +24719,7 @@
     </row>
     <row r="119" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A119" s="16" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B119" s="17">
         <v>20</v>
@@ -24757,7 +24763,7 @@
     </row>
     <row r="120" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A120" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B120" s="23">
         <v>1</v>
@@ -24801,7 +24807,7 @@
     </row>
     <row r="121" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A121" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B121" s="24">
         <v>2</v>
@@ -24845,7 +24851,7 @@
     </row>
     <row r="122" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A122" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B122" s="23">
         <v>3</v>
@@ -24889,7 +24895,7 @@
     </row>
     <row r="123" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A123" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B123" s="24">
         <v>4</v>
@@ -24933,7 +24939,7 @@
     </row>
     <row r="124" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A124" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B124" s="23">
         <v>5</v>
@@ -24977,7 +24983,7 @@
     </row>
     <row r="125" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A125" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B125" s="24">
         <v>6</v>
@@ -25021,7 +25027,7 @@
     </row>
     <row r="126" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A126" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B126" s="23">
         <v>7</v>
@@ -25065,7 +25071,7 @@
     </row>
     <row r="127" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A127" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B127" s="24">
         <v>8</v>
@@ -25109,7 +25115,7 @@
     </row>
     <row r="128" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A128" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B128" s="23">
         <v>9</v>
@@ -25153,7 +25159,7 @@
     </row>
     <row r="129" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A129" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B129" s="24">
         <v>10</v>
@@ -25197,7 +25203,7 @@
     </row>
     <row r="130" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A130" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B130" s="23">
         <v>11</v>
@@ -25241,7 +25247,7 @@
     </row>
     <row r="131" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A131" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B131" s="24">
         <v>12</v>
@@ -25285,7 +25291,7 @@
     </row>
     <row r="132" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A132" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B132" s="23">
         <v>13</v>
@@ -25329,7 +25335,7 @@
     </row>
     <row r="133" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A133" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B133" s="24">
         <v>14</v>
@@ -25373,7 +25379,7 @@
     </row>
     <row r="134" ht="14.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A134" s="16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B134" s="23">
         <v>15</v>

</xml_diff>